<commit_message>
Add ad spend and fixed average price to the cost model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DNFWtABRwmefxWQhJgZ3SK
</commit_message>
<xml_diff>
--- a/car-wash/finance/التكلفة-التشغيلية.xlsx
+++ b/car-wash/finance/التكلفة-التشغيلية.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
   <si>
     <t xml:space="preserve">Big Bubbles — نموذج التكلفة التشغيلية الشهرية</t>
   </si>
@@ -58,10 +58,19 @@
     <t xml:space="preserve">عدد العمال</t>
   </si>
   <si>
+    <t xml:space="preserve">السكن والإقامة ضمن الراتب</t>
+  </si>
+  <si>
     <t xml:space="preserve">راتب العامل (د.ك)</t>
   </si>
   <si>
-    <t xml:space="preserve">2) توزيع الباقات (نسبة من السيارات)</t>
+    <t xml:space="preserve">الإعلانات الشهرية (د.ك)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سوشال ميديا — بالكثير</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2) توزيع الباقات — للمواد ولو ما حطيت متوسط سعر</t>
   </si>
   <si>
     <t xml:space="preserve">الباقة</t>
@@ -142,10 +151,13 @@
     <t xml:space="preserve">✅ التكلفة التشغيلية الشهرية</t>
   </si>
   <si>
+    <t xml:space="preserve">📣 الإعلانات</t>
+  </si>
+  <si>
     <t xml:space="preserve">4) الدخل والربح (تقديري)</t>
   </si>
   <si>
-    <t xml:space="preserve">متوسط سعر الغسلة</t>
+    <t xml:space="preserve">متوسط سعر الغسلة المستخدم</t>
   </si>
   <si>
     <t xml:space="preserve">الدخل الشهري</t>
@@ -163,7 +175,13 @@
     <t xml:space="preserve">نقطة التعادل (سيارات باليوم — المجموع)</t>
   </si>
   <si>
-    <t xml:space="preserve">مو محسوب: صيانة السيارات، التأمين والتسجيل، سكن ومعيشة وإقامات العمال، الإعلانات، الجوالات، استهلاك المعدات.</t>
+    <t xml:space="preserve">متوسط سعر الغسلة — رقم ثابت (اختياري)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">امسحه عشان يتحسب من توزيع الباقات</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مو محسوب: الصيانة (السيارات تحت الكفالة) والتأمين (جاهز) — يتغير بعد انتهاء الكفالة. الجوالات واستهلاك المكاين.</t>
   </si>
 </sst>
 </file>
@@ -675,7 +693,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -762,42 +780,55 @@
       <c r="B10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="7"/>
+      <c r="C10" s="7" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>160</v>
       </c>
       <c r="C11" s="7"/>
     </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B15" s="11" t="n">
         <v>0.5</v>
@@ -811,7 +842,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>0.3</v>
@@ -825,7 +856,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B17" s="11" t="n">
         <v>0.15</v>
@@ -839,7 +870,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B18" s="11" t="n">
         <v>0.05</v>
@@ -853,7 +884,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B19" s="13" t="n">
         <f aca="false">SUM(B15:B18)</f>
@@ -862,14 +893,14 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B22" s="14" t="n">
         <f aca="false">B5*B6*B7</f>
@@ -879,7 +910,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B23" s="15" t="n">
         <f aca="false">SUMPRODUCT(B15:B18,D15:D18)</f>
@@ -889,7 +920,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B24" s="15" t="n">
         <f aca="false">B22*B23</f>
@@ -899,7 +930,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B25" s="15" t="n">
         <f aca="false">B5*B8*B7</f>
@@ -909,7 +940,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B26" s="15" t="n">
         <f aca="false">B5*B9*B7</f>
@@ -919,7 +950,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B27" s="15" t="n">
         <f aca="false">B10*B11</f>
@@ -929,76 +960,97 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B28" s="17" t="n">
-        <f aca="false">B24+B25+B26+B27</f>
-        <v>1182.88</v>
+        <f aca="false">B24+B25+B26+B27+B29</f>
+        <v>1282.88</v>
       </c>
       <c r="C28" s="16"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="15" t="n">
+        <f aca="false">B12</f>
+        <v>100</v>
+      </c>
+      <c r="C29" s="7"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B31" s="15" t="n">
-        <f aca="false">SUMPRODUCT(B15:B18,E15:E18)</f>
-        <v>8.925</v>
+        <f aca="false">IF(B36="",SUMPRODUCT(B15:B18,E15:E18),B36)</f>
+        <v>6</v>
       </c>
       <c r="C31" s="7"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B32" s="15" t="n">
         <f aca="false">B22*B31</f>
-        <v>3712.8</v>
+        <v>2496</v>
       </c>
       <c r="C32" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B33" s="17" t="n">
         <f aca="false">B32-B28</f>
-        <v>2529.92</v>
+        <v>1213.12</v>
       </c>
       <c r="C33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B34" s="8" t="n">
-        <f aca="false">(B25+B26+B27)/(B31-B23)</f>
-        <v>113.739545997611</v>
+        <f aca="false">(B25+B26+B27+B29)/(B31-B23)</f>
+        <v>193.204775022957</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B34/B7</f>
-        <v>4.37459792298502</v>
+        <v>7.43095288549834</v>
       </c>
       <c r="C35" s="7"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="18" t="s">
-        <v>38</v>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>